<commit_message>
Update syllabus processing scripts and documentation
</commit_message>
<xml_diff>
--- a/syllabus_books/R25_ECE_syllabus_courses_list.xlsx
+++ b/syllabus_books/R25_ECE_syllabus_courses_list.xlsx
@@ -432,11 +432,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="59" customWidth="1" min="2" max="2"/>
+    <col width="37" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="3" customWidth="1" min="4" max="4"/>
     <col width="3" customWidth="1" min="5" max="5"/>
@@ -495,7 +495,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Semiconductor Physics</t>
+          <t>ENGINEERING ELECTROMAGNETICS</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -513,10 +513,10 @@
         <v>2</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -527,7 +527,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Fundamentals of Semiconductor Physics for VLSI Laboratory</t>
+          <t>Digital Signal and Image Processing</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="D3" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E3" s="4" t="n">
         <v>0</v>
@@ -548,39 +548,7 @@
         <v>0</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>ECE002</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Course 2</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>PCM</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>